<commit_message>
Add initial DRF API and update RDO export
</commit_message>
<xml_diff>
--- a/assets/templates/modelo-de-diario-de-obras-2-0.xlsx
+++ b/assets/templates/modelo-de-diario-de-obras-2-0.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Meu Drive\SPATE - Drive\Arquivo 2025\Caltech\Palatium\Diário de obras\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\obrasys\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9BEC7C3-1857-4701-A130-39FDE0FF7885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388D11A8-1DF8-45B0-B118-F4966DBF27C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="15000" tabRatio="489" firstSheet="2" activeTab="3" xr2:uid="{87EA5CAA-EC54-48D1-96B5-889CC80A9EB0}"/>
   </bookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="111">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -405,9 +405,6 @@
     <t>Dia da semana</t>
   </si>
   <si>
-    <t xml:space="preserve">   D          S          T          Q          Q          S          S</t>
-  </si>
-  <si>
     <t>Responsável</t>
   </si>
   <si>
@@ -460,9 +457,6 @@
   </si>
   <si>
     <t>Quantidade utilizada</t>
-  </si>
-  <si>
-    <t>Equipamentos utilizados</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -485,12 +479,6 @@
     <t>Instalação dos tubos multicamadas e conexões</t>
   </si>
   <si>
-    <t>Anatonio Valdir</t>
-  </si>
-  <si>
-    <t>Paulinha</t>
-  </si>
-  <si>
     <t>Diário de Obra</t>
   </si>
   <si>
@@ -527,9 +515,6 @@
     <t>Apartamento modelo (apenas as localizadas nas paredes existentes)</t>
   </si>
   <si>
-    <t>intalação das caixas 4x2 de tomada e interruptores</t>
-  </si>
-  <si>
     <t xml:space="preserve">CAIXA DE PVC RETANGULAR 4"x2" </t>
   </si>
   <si>
@@ -548,13 +533,25 @@
     <t>ELETRODUTO PVC RÍGIDO ROSCÁVEL, CLASSE B, NBR-15465,  Ф 3/4" x 3,0m</t>
   </si>
   <si>
-    <t>Fixação das caixas octogonais de passagem</t>
-  </si>
-  <si>
     <t xml:space="preserve">Apartamento modelo </t>
   </si>
   <si>
-    <t>Fixação de eletrodutos</t>
+    <t>Equipe</t>
+  </si>
+  <si>
+    <t>Quantidade</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Atividade/Serviço executado</t>
+  </si>
+  <si>
+    <t>Disciplina</t>
+  </si>
+  <si>
+    <t>Materiais utilizados</t>
   </si>
 </sst>
 </file>
@@ -565,7 +562,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="48" x14ac:knownFonts="1">
+  <fonts count="49" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -851,6 +848,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -926,7 +929,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="46">
     <border>
       <left/>
       <right/>
@@ -1431,6 +1434,58 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF292F4B"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF292F4B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF292F4B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF292F4B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF292F4B"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF292F4B"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1443,7 +1498,7 @@
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="146">
+  <cellXfs count="158">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1579,6 +1634,15 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
@@ -1632,174 +1696,114 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1821,6 +1825,9 @@
     <xf numFmtId="0" fontId="38" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1839,20 +1846,104 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -2098,511 +2189,6 @@
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>304800</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>371475</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Retângulo 7">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CE13B3D2-CE06-4559-A1D8-D82EAFAB998F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3543300" y="1895475"/>
-          <a:ext cx="161925" cy="161925"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:sysClr val="window" lastClr="FFFFFF"/>
-        </a:solidFill>
-        <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="tx1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>571500</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Retângulo 10">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7AB3068F-2ED1-409B-9B60-CF1A265484B5}"/>
-            </a:ext>
-            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
-              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{CE13B3D2-CE06-4559-A1D8-D82EAFAB998F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3905250" y="1905000"/>
-          <a:ext cx="161925" cy="152400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:sysClr val="window" lastClr="FFFFFF"/>
-        </a:solidFill>
-        <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="tx1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" indent="0"/>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="lt1"/>
-            </a:solidFill>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>923925</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1087755</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="Retângulo 11">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1799336-2346-4C3F-AC09-0B42AA457280}"/>
-            </a:ext>
-            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
-              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{7AB3068F-2ED1-409B-9B60-CF1A265484B5}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4343400" y="2057400"/>
-          <a:ext cx="163830" cy="152400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:sysClr val="window" lastClr="FFFFFF"/>
-        </a:solidFill>
-        <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="tx1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" indent="0"/>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="lt1"/>
-            </a:solidFill>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1287780</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1455420</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="Retângulo 12">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{131354C0-FF04-45C6-A87C-BA7DEAF79060}"/>
-            </a:ext>
-            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
-              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{F1799336-2346-4C3F-AC09-0B42AA457280}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4707255" y="2066925"/>
-          <a:ext cx="167640" cy="152400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:sysClr val="window" lastClr="FFFFFF"/>
-        </a:solidFill>
-        <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="tx1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" indent="0"/>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="lt1"/>
-            </a:solidFill>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1657350</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1821180</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="6" name="Retângulo 13">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7BFBE410-BABA-4F22-9C8B-0EC9CCCF1C5F}"/>
-            </a:ext>
-            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
-              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{131354C0-FF04-45C6-A87C-BA7DEAF79060}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5076825" y="2057400"/>
-          <a:ext cx="163830" cy="161925"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="tx1"/>
-        </a:solidFill>
-        <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="tx1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" indent="0"/>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="lt1"/>
-            </a:solidFill>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>78105</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>243840</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="Retângulo 14">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{26A9E8A0-A693-4ACD-BA00-2DC2FD0A2E1C}"/>
-            </a:ext>
-            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
-              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{7BFBE410-BABA-4F22-9C8B-0EC9CCCF1C5F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5421630" y="2066925"/>
-          <a:ext cx="165735" cy="161925"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:sysClr val="window" lastClr="FFFFFF"/>
-        </a:solidFill>
-        <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="tx1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>415290</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>569595</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="8" name="Retângulo 15">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C3D6267-650E-427C-9843-9D8A76034828}"/>
-            </a:ext>
-            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
-              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{26A9E8A0-A693-4ACD-BA00-2DC2FD0A2E1C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5758815" y="2076450"/>
-          <a:ext cx="154305" cy="152400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:sysClr val="window" lastClr="FFFFFF"/>
-        </a:solidFill>
-        <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="tx1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -2612,9 +2198,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>893445</xdr:colOff>
+      <xdr:colOff>897255</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>15240</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2689,9 +2275,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1047750</xdr:colOff>
+      <xdr:colOff>1043940</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:rowOff>91440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2766,7 +2352,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1236345</xdr:colOff>
+      <xdr:colOff>1240155</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -2843,7 +2429,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>169545</xdr:colOff>
+      <xdr:colOff>173355</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -3319,22 +2905,22 @@
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="56" t="s">
+      <c r="B1" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="57"/>
-      <c r="M1" s="57"/>
-      <c r="N1" s="57"/>
-      <c r="O1" s="57"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
       <c r="P1" s="4"/>
       <c r="Q1" s="4"/>
       <c r="R1" s="4"/>
@@ -3344,20 +2930,20 @@
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="57"/>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57"/>
-      <c r="L2" s="57"/>
-      <c r="M2" s="57"/>
-      <c r="N2" s="57"/>
-      <c r="O2" s="57"/>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="I2" s="60"/>
+      <c r="J2" s="60"/>
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="M2" s="60"/>
+      <c r="N2" s="60"/>
+      <c r="O2" s="60"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
@@ -3386,105 +2972,105 @@
     </row>
     <row r="4" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="8"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
-      <c r="I4" s="58"/>
-      <c r="J4" s="58"/>
-      <c r="K4" s="58"/>
-      <c r="L4" s="58"/>
-      <c r="M4" s="58"/>
-      <c r="N4" s="58"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
+      <c r="G4" s="61"/>
+      <c r="H4" s="61"/>
+      <c r="I4" s="61"/>
+      <c r="J4" s="61"/>
+      <c r="K4" s="61"/>
+      <c r="L4" s="61"/>
+      <c r="M4" s="61"/>
+      <c r="N4" s="61"/>
       <c r="O4" s="8"/>
     </row>
     <row r="5" spans="1:19" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="8"/>
-      <c r="C5" s="59" t="s">
+      <c r="C5" s="62" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="59"/>
-      <c r="L5" s="59"/>
-      <c r="M5" s="59"/>
-      <c r="N5" s="59"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
+      <c r="H5" s="62"/>
+      <c r="I5" s="62"/>
+      <c r="J5" s="62"/>
+      <c r="K5" s="62"/>
+      <c r="L5" s="62"/>
+      <c r="M5" s="62"/>
+      <c r="N5" s="62"/>
       <c r="O5" s="8"/>
     </row>
     <row r="6" spans="1:19" ht="261.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="8"/>
       <c r="C6" s="9"/>
-      <c r="D6" s="66" t="s">
+      <c r="D6" s="69" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
-      <c r="G6" s="66"/>
-      <c r="H6" s="66"/>
-      <c r="I6" s="66"/>
-      <c r="J6" s="66"/>
-      <c r="K6" s="66"/>
-      <c r="L6" s="66"/>
-      <c r="M6" s="66"/>
-      <c r="N6" s="66"/>
-      <c r="O6" s="66"/>
+      <c r="E6" s="69"/>
+      <c r="F6" s="69"/>
+      <c r="G6" s="69"/>
+      <c r="H6" s="69"/>
+      <c r="I6" s="69"/>
+      <c r="J6" s="69"/>
+      <c r="K6" s="69"/>
+      <c r="L6" s="69"/>
+      <c r="M6" s="69"/>
+      <c r="N6" s="69"/>
+      <c r="O6" s="69"/>
     </row>
     <row r="7" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C7" s="60"/>
-      <c r="D7" s="60"/>
-      <c r="E7" s="60"/>
-      <c r="F7" s="60"/>
-      <c r="G7" s="60"/>
-      <c r="H7" s="60"/>
-      <c r="I7" s="60"/>
-      <c r="J7" s="60"/>
-      <c r="K7" s="60"/>
-      <c r="L7" s="60"/>
-      <c r="M7" s="60"/>
-      <c r="N7" s="60"/>
+      <c r="C7" s="63"/>
+      <c r="D7" s="63"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="63"/>
+      <c r="G7" s="63"/>
+      <c r="H7" s="63"/>
+      <c r="I7" s="63"/>
+      <c r="J7" s="63"/>
+      <c r="K7" s="63"/>
+      <c r="L7" s="63"/>
+      <c r="M7" s="63"/>
+      <c r="N7" s="63"/>
     </row>
     <row r="8" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="62" t="s">
+      <c r="B8" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
-      <c r="G8" s="62"/>
-      <c r="H8" s="62"/>
-      <c r="I8" s="62"/>
-      <c r="J8" s="62"/>
-      <c r="K8" s="62"/>
-      <c r="L8" s="62"/>
-      <c r="M8" s="62"/>
-      <c r="N8" s="62"/>
-      <c r="O8" s="62"/>
+      <c r="C8" s="65"/>
+      <c r="D8" s="65"/>
+      <c r="E8" s="65"/>
+      <c r="F8" s="65"/>
+      <c r="G8" s="65"/>
+      <c r="H8" s="65"/>
+      <c r="I8" s="65"/>
+      <c r="J8" s="65"/>
+      <c r="K8" s="65"/>
+      <c r="L8" s="65"/>
+      <c r="M8" s="65"/>
+      <c r="N8" s="65"/>
+      <c r="O8" s="65"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="63"/>
-      <c r="D9" s="63"/>
-      <c r="E9" s="63"/>
-      <c r="F9" s="63"/>
-      <c r="G9" s="63"/>
-      <c r="H9" s="63"/>
-      <c r="I9" s="63"/>
-      <c r="J9" s="63"/>
-      <c r="K9" s="63"/>
-      <c r="L9" s="63"/>
-      <c r="M9" s="63"/>
-      <c r="N9" s="63"/>
-      <c r="O9" s="63"/>
+      <c r="C9" s="66"/>
+      <c r="D9" s="66"/>
+      <c r="E9" s="66"/>
+      <c r="F9" s="66"/>
+      <c r="G9" s="66"/>
+      <c r="H9" s="66"/>
+      <c r="I9" s="66"/>
+      <c r="J9" s="66"/>
+      <c r="K9" s="66"/>
+      <c r="L9" s="66"/>
+      <c r="M9" s="66"/>
+      <c r="N9" s="66"/>
+      <c r="O9" s="66"/>
     </row>
     <row r="10" spans="1:19" ht="4.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="44"/>
@@ -3503,40 +3089,40 @@
       <c r="O10" s="47"/>
     </row>
     <row r="11" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="64" t="s">
+      <c r="B11" s="67" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="64"/>
-      <c r="D11" s="64"/>
-      <c r="E11" s="64"/>
-      <c r="F11" s="64"/>
-      <c r="G11" s="64"/>
-      <c r="H11" s="64"/>
-      <c r="I11" s="64"/>
-      <c r="J11" s="64"/>
-      <c r="K11" s="64"/>
-      <c r="L11" s="64"/>
-      <c r="M11" s="64"/>
-      <c r="N11" s="64"/>
-      <c r="O11" s="64"/>
+      <c r="C11" s="67"/>
+      <c r="D11" s="67"/>
+      <c r="E11" s="67"/>
+      <c r="F11" s="67"/>
+      <c r="G11" s="67"/>
+      <c r="H11" s="67"/>
+      <c r="I11" s="67"/>
+      <c r="J11" s="67"/>
+      <c r="K11" s="67"/>
+      <c r="L11" s="67"/>
+      <c r="M11" s="67"/>
+      <c r="N11" s="67"/>
+      <c r="O11" s="67"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="63" t="s">
+      <c r="B12" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="63"/>
-      <c r="D12" s="63"/>
-      <c r="E12" s="63"/>
-      <c r="F12" s="63"/>
-      <c r="G12" s="63"/>
-      <c r="H12" s="63"/>
-      <c r="I12" s="63"/>
-      <c r="J12" s="63"/>
-      <c r="K12" s="63"/>
-      <c r="L12" s="63"/>
-      <c r="M12" s="63"/>
-      <c r="N12" s="63"/>
-      <c r="O12" s="63"/>
+      <c r="C12" s="66"/>
+      <c r="D12" s="66"/>
+      <c r="E12" s="66"/>
+      <c r="F12" s="66"/>
+      <c r="G12" s="66"/>
+      <c r="H12" s="66"/>
+      <c r="I12" s="66"/>
+      <c r="J12" s="66"/>
+      <c r="K12" s="66"/>
+      <c r="L12" s="66"/>
+      <c r="M12" s="66"/>
+      <c r="N12" s="66"/>
+      <c r="O12" s="66"/>
     </row>
     <row r="13" spans="1:19" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B13" s="48"/>
@@ -3555,88 +3141,88 @@
       <c r="O13" s="43"/>
     </row>
     <row r="14" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="65" t="s">
+      <c r="B14" s="68" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="65"/>
-      <c r="D14" s="65"/>
-      <c r="E14" s="65"/>
-      <c r="F14" s="65"/>
-      <c r="G14" s="65"/>
-      <c r="H14" s="65"/>
-      <c r="I14" s="65"/>
-      <c r="J14" s="65"/>
-      <c r="K14" s="65"/>
-      <c r="L14" s="65"/>
-      <c r="M14" s="65"/>
-      <c r="N14" s="65"/>
-      <c r="O14" s="65"/>
+      <c r="C14" s="68"/>
+      <c r="D14" s="68"/>
+      <c r="E14" s="68"/>
+      <c r="F14" s="68"/>
+      <c r="G14" s="68"/>
+      <c r="H14" s="68"/>
+      <c r="I14" s="68"/>
+      <c r="J14" s="68"/>
+      <c r="K14" s="68"/>
+      <c r="L14" s="68"/>
+      <c r="M14" s="68"/>
+      <c r="N14" s="68"/>
+      <c r="O14" s="68"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="65"/>
-      <c r="C15" s="65"/>
-      <c r="D15" s="65"/>
-      <c r="E15" s="65"/>
-      <c r="F15" s="65"/>
-      <c r="G15" s="65"/>
-      <c r="H15" s="65"/>
-      <c r="I15" s="65"/>
-      <c r="J15" s="65"/>
-      <c r="K15" s="65"/>
-      <c r="L15" s="65"/>
-      <c r="M15" s="65"/>
-      <c r="N15" s="65"/>
-      <c r="O15" s="65"/>
+      <c r="B15" s="68"/>
+      <c r="C15" s="68"/>
+      <c r="D15" s="68"/>
+      <c r="E15" s="68"/>
+      <c r="F15" s="68"/>
+      <c r="G15" s="68"/>
+      <c r="H15" s="68"/>
+      <c r="I15" s="68"/>
+      <c r="J15" s="68"/>
+      <c r="K15" s="68"/>
+      <c r="L15" s="68"/>
+      <c r="M15" s="68"/>
+      <c r="N15" s="68"/>
+      <c r="O15" s="68"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="B16" s="61"/>
-      <c r="C16" s="61"/>
-      <c r="D16" s="61"/>
-      <c r="E16" s="61"/>
-      <c r="F16" s="61"/>
-      <c r="G16" s="61"/>
-      <c r="H16" s="61"/>
-      <c r="I16" s="61"/>
-      <c r="J16" s="61"/>
-      <c r="K16" s="61"/>
-      <c r="L16" s="61"/>
-      <c r="M16" s="61"/>
-      <c r="N16" s="61"/>
-      <c r="O16" s="61"/>
+      <c r="B16" s="64"/>
+      <c r="C16" s="64"/>
+      <c r="D16" s="64"/>
+      <c r="E16" s="64"/>
+      <c r="F16" s="64"/>
+      <c r="G16" s="64"/>
+      <c r="H16" s="64"/>
+      <c r="I16" s="64"/>
+      <c r="J16" s="64"/>
+      <c r="K16" s="64"/>
+      <c r="L16" s="64"/>
+      <c r="M16" s="64"/>
+      <c r="N16" s="64"/>
+      <c r="O16" s="64"/>
     </row>
     <row r="17" spans="2:15" ht="24.6" x14ac:dyDescent="0.3">
       <c r="B17" s="12"/>
-      <c r="C17" s="67" t="s">
+      <c r="C17" s="70" t="s">
         <v>9</v>
       </c>
-      <c r="D17" s="68"/>
-      <c r="E17" s="68"/>
-      <c r="F17" s="68"/>
-      <c r="G17" s="68"/>
-      <c r="H17" s="68"/>
-      <c r="I17" s="68"/>
-      <c r="J17" s="68"/>
-      <c r="K17" s="68"/>
-      <c r="L17" s="68"/>
-      <c r="M17" s="68"/>
+      <c r="D17" s="71"/>
+      <c r="E17" s="71"/>
+      <c r="F17" s="71"/>
+      <c r="G17" s="71"/>
+      <c r="H17" s="71"/>
+      <c r="I17" s="71"/>
+      <c r="J17" s="71"/>
+      <c r="K17" s="71"/>
+      <c r="L17" s="71"/>
+      <c r="M17" s="71"/>
       <c r="N17" s="12"/>
       <c r="O17" s="12"/>
     </row>
     <row r="18" spans="2:15" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
-      <c r="D18" s="53" t="s">
+      <c r="D18" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="E18" s="54"/>
-      <c r="F18" s="54"/>
-      <c r="G18" s="54"/>
-      <c r="H18" s="54"/>
-      <c r="I18" s="54"/>
-      <c r="J18" s="54"/>
-      <c r="K18" s="54"/>
-      <c r="L18" s="54"/>
-      <c r="M18" s="54"/>
+      <c r="E18" s="57"/>
+      <c r="F18" s="57"/>
+      <c r="G18" s="57"/>
+      <c r="H18" s="57"/>
+      <c r="I18" s="57"/>
+      <c r="J18" s="57"/>
+      <c r="K18" s="57"/>
+      <c r="L18" s="57"/>
+      <c r="M18" s="57"/>
       <c r="N18" s="12"/>
       <c r="O18" s="12"/>
     </row>
@@ -3659,16 +3245,16 @@
     <row r="20" spans="2:15" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="12"/>
       <c r="C20" s="15"/>
-      <c r="D20" s="55" t="s">
+      <c r="D20" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="E20" s="55"/>
-      <c r="F20" s="55"/>
-      <c r="G20" s="55"/>
-      <c r="H20" s="55"/>
-      <c r="I20" s="55"/>
-      <c r="J20" s="55"/>
-      <c r="K20" s="55"/>
+      <c r="E20" s="58"/>
+      <c r="F20" s="58"/>
+      <c r="G20" s="58"/>
+      <c r="H20" s="58"/>
+      <c r="I20" s="58"/>
+      <c r="J20" s="58"/>
+      <c r="K20" s="58"/>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
       <c r="N20" s="12"/>
@@ -3765,22 +3351,22 @@
       <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="69" t="s">
+      <c r="B1" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+      <c r="O1" s="73"/>
       <c r="P1" s="4"/>
       <c r="Q1" s="4"/>
       <c r="R1" s="4"/>
@@ -3788,20 +3374,20 @@
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="73"/>
+      <c r="M2" s="73"/>
+      <c r="N2" s="73"/>
+      <c r="O2" s="73"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
@@ -3830,85 +3416,85 @@
     </row>
     <row r="4" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="8"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
-      <c r="I4" s="58"/>
-      <c r="J4" s="58"/>
-      <c r="K4" s="58"/>
-      <c r="L4" s="58"/>
-      <c r="M4" s="58"/>
-      <c r="N4" s="58"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
+      <c r="G4" s="61"/>
+      <c r="H4" s="61"/>
+      <c r="I4" s="61"/>
+      <c r="J4" s="61"/>
+      <c r="K4" s="61"/>
+      <c r="L4" s="61"/>
+      <c r="M4" s="61"/>
+      <c r="N4" s="61"/>
       <c r="O4" s="8"/>
     </row>
     <row r="5" spans="1:19" ht="92.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="8"/>
-      <c r="C5" s="59" t="s">
+      <c r="C5" s="62" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="59"/>
-      <c r="L5" s="59"/>
-      <c r="M5" s="59"/>
-      <c r="N5" s="59"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
+      <c r="H5" s="62"/>
+      <c r="I5" s="62"/>
+      <c r="J5" s="62"/>
+      <c r="K5" s="62"/>
+      <c r="L5" s="62"/>
+      <c r="M5" s="62"/>
+      <c r="N5" s="62"/>
       <c r="O5" s="8"/>
     </row>
     <row r="6" spans="1:19" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="8"/>
       <c r="C6" s="9"/>
-      <c r="D6" s="66" t="s">
+      <c r="D6" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="71"/>
-      <c r="F6" s="71"/>
-      <c r="G6" s="71"/>
-      <c r="H6" s="71"/>
-      <c r="I6" s="71"/>
-      <c r="J6" s="71"/>
-      <c r="K6" s="71"/>
-      <c r="L6" s="71"/>
-      <c r="M6" s="71"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
+      <c r="G6" s="74"/>
+      <c r="H6" s="74"/>
+      <c r="I6" s="74"/>
+      <c r="J6" s="74"/>
+      <c r="K6" s="74"/>
+      <c r="L6" s="74"/>
+      <c r="M6" s="74"/>
       <c r="N6" s="8"/>
       <c r="O6" s="8"/>
     </row>
     <row r="7" spans="1:19" ht="230.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="8"/>
       <c r="C7" s="10"/>
-      <c r="D7" s="71"/>
-      <c r="E7" s="71"/>
-      <c r="F7" s="71"/>
-      <c r="G7" s="71"/>
-      <c r="H7" s="71"/>
-      <c r="I7" s="71"/>
-      <c r="J7" s="71"/>
-      <c r="K7" s="71"/>
-      <c r="L7" s="71"/>
-      <c r="M7" s="71"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
+      <c r="F7" s="74"/>
+      <c r="G7" s="74"/>
+      <c r="H7" s="74"/>
+      <c r="I7" s="74"/>
+      <c r="J7" s="74"/>
+      <c r="K7" s="74"/>
+      <c r="L7" s="74"/>
+      <c r="M7" s="74"/>
       <c r="N7" s="11"/>
       <c r="O7" s="8"/>
     </row>
     <row r="8" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C8" s="60"/>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="60"/>
-      <c r="G8" s="60"/>
-      <c r="H8" s="60"/>
-      <c r="I8" s="60"/>
-      <c r="J8" s="60"/>
-      <c r="K8" s="60"/>
-      <c r="L8" s="60"/>
-      <c r="M8" s="60"/>
-      <c r="N8" s="60"/>
+      <c r="C8" s="63"/>
+      <c r="D8" s="63"/>
+      <c r="E8" s="63"/>
+      <c r="F8" s="63"/>
+      <c r="G8" s="63"/>
+      <c r="H8" s="63"/>
+      <c r="I8" s="63"/>
+      <c r="J8" s="63"/>
+      <c r="K8" s="63"/>
+      <c r="L8" s="63"/>
+      <c r="M8" s="63"/>
+      <c r="N8" s="63"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B9" s="7"/>
@@ -3959,87 +3545,87 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="80"/>
-      <c r="C1" s="80"/>
-      <c r="D1" s="80"/>
-      <c r="E1" s="80"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
       <c r="F1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="4.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="88" t="e" vm="1">
+      <c r="A3" s="95" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B3" s="89"/>
-      <c r="C3" s="82"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="84"/>
+      <c r="B3" s="96"/>
+      <c r="C3" s="89"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="91"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="88"/>
-      <c r="B4" s="89"/>
-      <c r="C4" s="94" t="s">
+      <c r="A4" s="95"/>
+      <c r="B4" s="96"/>
+      <c r="C4" s="76" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="95"/>
-      <c r="E4" s="96"/>
+      <c r="D4" s="77"/>
+      <c r="E4" s="78"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="88"/>
-      <c r="B5" s="89"/>
-      <c r="C5" s="97" t="s">
+      <c r="A5" s="95"/>
+      <c r="B5" s="96"/>
+      <c r="C5" s="81" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="98"/>
-      <c r="E5" s="99"/>
+      <c r="D5" s="82"/>
+      <c r="E5" s="83"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="88"/>
-      <c r="B6" s="89"/>
-      <c r="C6" s="77" t="s">
+      <c r="A6" s="95"/>
+      <c r="B6" s="96"/>
+      <c r="C6" s="84" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="78"/>
-      <c r="E6" s="79"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="86"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="88"/>
-      <c r="B7" s="89"/>
-      <c r="C7" s="85"/>
-      <c r="D7" s="86"/>
-      <c r="E7" s="87"/>
+      <c r="A7" s="95"/>
+      <c r="B7" s="96"/>
+      <c r="C7" s="92"/>
+      <c r="D7" s="93"/>
+      <c r="E7" s="94"/>
     </row>
     <row r="8" spans="1:6" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A8" s="90" t="s">
+      <c r="A8" s="97" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="90"/>
-      <c r="C8" s="91"/>
-      <c r="D8" s="91"/>
-      <c r="E8" s="91"/>
+      <c r="B8" s="97"/>
+      <c r="C8" s="98"/>
+      <c r="D8" s="98"/>
+      <c r="E8" s="98"/>
     </row>
     <row r="9" spans="1:6" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A9" s="92" t="s">
+      <c r="A9" s="99" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="92"/>
-      <c r="C9" s="92"/>
-      <c r="D9" s="92"/>
-      <c r="E9" s="92"/>
+      <c r="B9" s="99"/>
+      <c r="C9" s="99"/>
+      <c r="D9" s="99"/>
+      <c r="E9" s="99"/>
     </row>
     <row r="10" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="75"/>
-      <c r="C10" s="75"/>
-      <c r="D10" s="75"/>
-      <c r="E10" s="75"/>
+      <c r="B10" s="79"/>
+      <c r="C10" s="79"/>
+      <c r="D10" s="79"/>
+      <c r="E10" s="79"/>
     </row>
     <row r="11" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="36" t="s">
@@ -4049,8 +3635,8 @@
       <c r="C11" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="75"/>
-      <c r="E11" s="75"/>
+      <c r="D11" s="79"/>
+      <c r="E11" s="79"/>
     </row>
     <row r="12" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="36" t="s">
@@ -4060,17 +3646,17 @@
       <c r="C12" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="75"/>
-      <c r="E12" s="75"/>
+      <c r="D12" s="79"/>
+      <c r="E12" s="79"/>
     </row>
     <row r="13" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="75"/>
-      <c r="C13" s="75"/>
-      <c r="D13" s="75"/>
-      <c r="E13" s="75"/>
+      <c r="B13" s="79"/>
+      <c r="C13" s="79"/>
+      <c r="D13" s="79"/>
+      <c r="E13" s="79"/>
     </row>
     <row r="14" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="36" t="s">
@@ -4080,8 +3666,8 @@
       <c r="C14" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="75"/>
-      <c r="E14" s="75"/>
+      <c r="D14" s="79"/>
+      <c r="E14" s="79"/>
     </row>
     <row r="15" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="36" t="s">
@@ -4091,8 +3677,8 @@
       <c r="C15" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="75"/>
-      <c r="E15" s="75"/>
+      <c r="D15" s="79"/>
+      <c r="E15" s="79"/>
     </row>
     <row r="16" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="36" t="s">
@@ -4102,35 +3688,35 @@
       <c r="C16" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="75"/>
-      <c r="E16" s="75"/>
+      <c r="D16" s="79"/>
+      <c r="E16" s="79"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="75"/>
-      <c r="C17" s="75"/>
-      <c r="D17" s="75"/>
-      <c r="E17" s="75"/>
+      <c r="B17" s="79"/>
+      <c r="C17" s="79"/>
+      <c r="D17" s="79"/>
+      <c r="E17" s="79"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A18" s="72" t="s">
+      <c r="A18" s="80" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="72"/>
-      <c r="C18" s="72"/>
-      <c r="D18" s="72"/>
-      <c r="E18" s="72"/>
+      <c r="B18" s="80"/>
+      <c r="C18" s="80"/>
+      <c r="D18" s="80"/>
+      <c r="E18" s="80"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="75"/>
-      <c r="C19" s="75"/>
-      <c r="D19" s="75"/>
-      <c r="E19" s="75"/>
+      <c r="B19" s="79"/>
+      <c r="C19" s="79"/>
+      <c r="D19" s="79"/>
+      <c r="E19" s="79"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="36" t="s">
@@ -4140,17 +3726,17 @@
       <c r="C20" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="75"/>
-      <c r="E20" s="75"/>
+      <c r="D20" s="79"/>
+      <c r="E20" s="79"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="75"/>
-      <c r="C21" s="75"/>
-      <c r="D21" s="75"/>
-      <c r="E21" s="75"/>
+      <c r="B21" s="79"/>
+      <c r="C21" s="79"/>
+      <c r="D21" s="79"/>
+      <c r="E21" s="79"/>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="36" t="s">
@@ -4160,8 +3746,8 @@
       <c r="C22" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="D22" s="75"/>
-      <c r="E22" s="75"/>
+      <c r="D22" s="79"/>
+      <c r="E22" s="79"/>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="36" t="s">
@@ -4171,8 +3757,8 @@
       <c r="C23" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="75"/>
-      <c r="E23" s="75"/>
+      <c r="D23" s="79"/>
+      <c r="E23" s="79"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="36" t="s">
@@ -4182,76 +3768,76 @@
       <c r="C24" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="D24" s="75"/>
-      <c r="E24" s="75"/>
+      <c r="D24" s="79"/>
+      <c r="E24" s="79"/>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="75"/>
-      <c r="C25" s="75"/>
-      <c r="D25" s="75"/>
-      <c r="E25" s="75"/>
+      <c r="B25" s="79"/>
+      <c r="C25" s="79"/>
+      <c r="D25" s="79"/>
+      <c r="E25" s="79"/>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A26" s="81" t="s">
+      <c r="A26" s="88" t="s">
         <v>37</v>
       </c>
-      <c r="B26" s="72"/>
-      <c r="C26" s="72"/>
-      <c r="D26" s="72"/>
-      <c r="E26" s="72"/>
+      <c r="B26" s="80"/>
+      <c r="C26" s="80"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="80"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="B27" s="75" t="s">
-        <v>94</v>
-      </c>
-      <c r="C27" s="75"/>
-      <c r="D27" s="75"/>
-      <c r="E27" s="75"/>
+      <c r="B27" s="79" t="s">
+        <v>90</v>
+      </c>
+      <c r="C27" s="79"/>
+      <c r="D27" s="79"/>
+      <c r="E27" s="79"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="36" t="s">
         <v>26</v>
       </c>
       <c r="B28" s="37" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C28" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="D28" s="75" t="s">
-        <v>96</v>
-      </c>
-      <c r="E28" s="75"/>
+      <c r="D28" s="79" t="s">
+        <v>92</v>
+      </c>
+      <c r="E28" s="79"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="36" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="37" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C29" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="D29" s="75" t="s">
-        <v>97</v>
-      </c>
-      <c r="E29" s="75"/>
+      <c r="D29" s="79" t="s">
+        <v>93</v>
+      </c>
+      <c r="E29" s="79"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="B30" s="75"/>
-      <c r="C30" s="75"/>
-      <c r="D30" s="75"/>
-      <c r="E30" s="75"/>
+      <c r="B30" s="79"/>
+      <c r="C30" s="79"/>
+      <c r="D30" s="79"/>
+      <c r="E30" s="79"/>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="36" t="s">
@@ -4261,28 +3847,28 @@
       <c r="C31" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="D31" s="75"/>
-      <c r="E31" s="75"/>
+      <c r="D31" s="79"/>
+      <c r="E31" s="79"/>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="B32" s="75" t="s">
-        <v>99</v>
-      </c>
-      <c r="C32" s="75"/>
-      <c r="D32" s="75"/>
-      <c r="E32" s="75"/>
+      <c r="B32" s="79" t="s">
+        <v>95</v>
+      </c>
+      <c r="C32" s="79"/>
+      <c r="D32" s="79"/>
+      <c r="E32" s="79"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="B33" s="75"/>
-      <c r="C33" s="75"/>
-      <c r="D33" s="75"/>
-      <c r="E33" s="75"/>
+      <c r="B33" s="79"/>
+      <c r="C33" s="79"/>
+      <c r="D33" s="79"/>
+      <c r="E33" s="79"/>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="36" t="s">
@@ -4291,38 +3877,38 @@
       <c r="B34" s="51">
         <v>46113</v>
       </c>
-      <c r="C34" s="93" t="s">
+      <c r="C34" s="75" t="s">
         <v>45</v>
       </c>
-      <c r="D34" s="93"/>
+      <c r="D34" s="75"/>
       <c r="E34" s="37"/>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A35" s="72" t="s">
+      <c r="A35" s="80" t="s">
         <v>37</v>
       </c>
-      <c r="B35" s="72"/>
-      <c r="C35" s="72"/>
-      <c r="D35" s="72"/>
-      <c r="E35" s="72"/>
+      <c r="B35" s="80"/>
+      <c r="C35" s="80"/>
+      <c r="D35" s="80"/>
+      <c r="E35" s="80"/>
     </row>
     <row r="36" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="B36" s="75"/>
-      <c r="C36" s="75"/>
-      <c r="D36" s="75"/>
-      <c r="E36" s="75"/>
+      <c r="B36" s="79"/>
+      <c r="C36" s="79"/>
+      <c r="D36" s="79"/>
+      <c r="E36" s="79"/>
     </row>
     <row r="37" spans="1:5" s="1" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="B37" s="75" t="s">
-        <v>91</v>
-      </c>
-      <c r="C37" s="75"/>
+      <c r="B37" s="79" t="s">
+        <v>87</v>
+      </c>
+      <c r="C37" s="79"/>
       <c r="D37" s="36" t="s">
         <v>48</v>
       </c>
@@ -4332,111 +3918,111 @@
       <c r="A38" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="B38" s="76" t="s">
-        <v>100</v>
-      </c>
-      <c r="C38" s="76"/>
+      <c r="B38" s="102" t="s">
+        <v>96</v>
+      </c>
+      <c r="C38" s="102"/>
       <c r="D38" s="39" t="s">
         <v>48</v>
       </c>
       <c r="E38" s="40"/>
     </row>
     <row r="39" spans="1:5" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A39" s="73" t="s">
+      <c r="A39" s="100" t="s">
         <v>49</v>
       </c>
-      <c r="B39" s="73"/>
-      <c r="C39" s="73"/>
-      <c r="D39" s="73"/>
-      <c r="E39" s="73"/>
+      <c r="B39" s="100"/>
+      <c r="C39" s="100"/>
+      <c r="D39" s="100"/>
+      <c r="E39" s="100"/>
     </row>
     <row r="40" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="75"/>
-      <c r="B40" s="75"/>
-      <c r="C40" s="75"/>
-      <c r="D40" s="75"/>
-      <c r="E40" s="75"/>
+      <c r="A40" s="79"/>
+      <c r="B40" s="79"/>
+      <c r="C40" s="79"/>
+      <c r="D40" s="79"/>
+      <c r="E40" s="79"/>
     </row>
     <row r="41" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="75"/>
-      <c r="B41" s="75"/>
-      <c r="C41" s="75"/>
-      <c r="D41" s="75"/>
-      <c r="E41" s="75"/>
+      <c r="A41" s="79"/>
+      <c r="B41" s="79"/>
+      <c r="C41" s="79"/>
+      <c r="D41" s="79"/>
+      <c r="E41" s="79"/>
     </row>
     <row r="42" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="75"/>
-      <c r="B42" s="75"/>
-      <c r="C42" s="75"/>
-      <c r="D42" s="75"/>
-      <c r="E42" s="75"/>
+      <c r="A42" s="79"/>
+      <c r="B42" s="79"/>
+      <c r="C42" s="79"/>
+      <c r="D42" s="79"/>
+      <c r="E42" s="79"/>
     </row>
     <row r="43" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="75"/>
-      <c r="B43" s="75"/>
-      <c r="C43" s="75"/>
-      <c r="D43" s="75"/>
-      <c r="E43" s="75"/>
+      <c r="A43" s="79"/>
+      <c r="B43" s="79"/>
+      <c r="C43" s="79"/>
+      <c r="D43" s="79"/>
+      <c r="E43" s="79"/>
     </row>
     <row r="44" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="75"/>
-      <c r="B44" s="75"/>
-      <c r="C44" s="75"/>
-      <c r="D44" s="75"/>
-      <c r="E44" s="75"/>
+      <c r="A44" s="79"/>
+      <c r="B44" s="79"/>
+      <c r="C44" s="79"/>
+      <c r="D44" s="79"/>
+      <c r="E44" s="79"/>
     </row>
     <row r="45" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="75"/>
-      <c r="B45" s="75"/>
-      <c r="C45" s="75"/>
-      <c r="D45" s="75"/>
-      <c r="E45" s="75"/>
+      <c r="A45" s="79"/>
+      <c r="B45" s="79"/>
+      <c r="C45" s="79"/>
+      <c r="D45" s="79"/>
+      <c r="E45" s="79"/>
     </row>
     <row r="46" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="75"/>
-      <c r="B46" s="75"/>
-      <c r="C46" s="75"/>
-      <c r="D46" s="75"/>
-      <c r="E46" s="75"/>
+      <c r="A46" s="79"/>
+      <c r="B46" s="79"/>
+      <c r="C46" s="79"/>
+      <c r="D46" s="79"/>
+      <c r="E46" s="79"/>
     </row>
     <row r="47" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="75"/>
-      <c r="B47" s="75"/>
-      <c r="C47" s="75"/>
-      <c r="D47" s="75"/>
-      <c r="E47" s="75"/>
+      <c r="A47" s="79"/>
+      <c r="B47" s="79"/>
+      <c r="C47" s="79"/>
+      <c r="D47" s="79"/>
+      <c r="E47" s="79"/>
     </row>
     <row r="48" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="75"/>
-      <c r="B48" s="75"/>
-      <c r="C48" s="75"/>
-      <c r="D48" s="75"/>
-      <c r="E48" s="75"/>
+      <c r="A48" s="79"/>
+      <c r="B48" s="79"/>
+      <c r="C48" s="79"/>
+      <c r="D48" s="79"/>
+      <c r="E48" s="79"/>
     </row>
     <row r="49" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="74" t="s">
+      <c r="A49" s="101" t="s">
         <v>50</v>
       </c>
-      <c r="B49" s="74"/>
-      <c r="C49" s="74"/>
-      <c r="D49" s="74"/>
-      <c r="E49" s="74"/>
+      <c r="B49" s="101"/>
+      <c r="C49" s="101"/>
+      <c r="D49" s="101"/>
+      <c r="E49" s="101"/>
     </row>
     <row r="50" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="36" t="s">
         <v>51</v>
       </c>
-      <c r="B50" s="75"/>
-      <c r="C50" s="75"/>
-      <c r="D50" s="75"/>
-      <c r="E50" s="75"/>
+      <c r="B50" s="79"/>
+      <c r="C50" s="79"/>
+      <c r="D50" s="79"/>
+      <c r="E50" s="79"/>
     </row>
     <row r="51" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="B51" s="75"/>
-      <c r="C51" s="75"/>
+      <c r="B51" s="79"/>
+      <c r="C51" s="79"/>
       <c r="D51" s="36" t="s">
         <v>48</v>
       </c>
@@ -4454,6 +4040,41 @@
     </row>
   </sheetData>
   <mergeCells count="51">
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="A3:B7"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="B10:E10"/>
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="D11:E11"/>
@@ -4470,41 +4091,6 @@
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="C5:E5"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="A3:B7"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B50:E50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="A45:E45"/>
-    <mergeCell ref="A43:E43"/>
-    <mergeCell ref="A47:E47"/>
-    <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A46:E46"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="A40:E40"/>
-    <mergeCell ref="A42:E42"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
   </mergeCells>
   <pageMargins left="0.78740157480314965" right="0.59055118110236227" top="0.59055118110236227" bottom="0.59055118110236227" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
@@ -4517,7 +4103,7 @@
     <tabColor rgb="FF292F4B"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="19" customWidth="1"/>
@@ -4530,63 +4116,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="127" t="s">
-        <v>90</v>
-      </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="127"/>
+      <c r="A1" s="109" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="109"/>
+      <c r="C1" s="109"/>
+      <c r="D1" s="109"/>
+      <c r="E1" s="109"/>
+      <c r="F1" s="109"/>
       <c r="G1" s="19" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="122" t="e" vm="1">
+      <c r="A2" s="118" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B2" s="122"/>
-      <c r="C2" s="122"/>
-      <c r="D2" s="101" t="s">
-        <v>84</v>
-      </c>
-      <c r="E2" s="102"/>
-      <c r="F2" s="103"/>
+      <c r="B2" s="118"/>
+      <c r="C2" s="118"/>
+      <c r="D2" s="137" t="s">
+        <v>82</v>
+      </c>
+      <c r="E2" s="138"/>
+      <c r="F2" s="139"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="122"/>
-      <c r="B3" s="122"/>
-      <c r="C3" s="122"/>
-      <c r="D3" s="104"/>
-      <c r="E3" s="105"/>
-      <c r="F3" s="106"/>
+      <c r="A3" s="118"/>
+      <c r="B3" s="118"/>
+      <c r="C3" s="118"/>
+      <c r="D3" s="140"/>
+      <c r="E3" s="141"/>
+      <c r="F3" s="142"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="122"/>
-      <c r="B4" s="122"/>
-      <c r="C4" s="122"/>
-      <c r="D4" s="107"/>
-      <c r="E4" s="108"/>
-      <c r="F4" s="109"/>
+      <c r="A4" s="118"/>
+      <c r="B4" s="118"/>
+      <c r="C4" s="118"/>
+      <c r="D4" s="143"/>
+      <c r="E4" s="144"/>
+      <c r="F4" s="145"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="122"/>
-      <c r="B5" s="122"/>
-      <c r="C5" s="122"/>
-      <c r="D5" s="135" t="s">
-        <v>93</v>
-      </c>
-      <c r="E5" s="136"/>
-      <c r="F5" s="137"/>
+      <c r="A5" s="118"/>
+      <c r="B5" s="118"/>
+      <c r="C5" s="118"/>
+      <c r="D5" s="119" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" s="120"/>
+      <c r="F5" s="121"/>
     </row>
     <row r="6" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="122"/>
-      <c r="B6" s="122"/>
-      <c r="C6" s="122"/>
-      <c r="D6" s="138"/>
-      <c r="E6" s="139"/>
-      <c r="F6" s="140"/>
+      <c r="A6" s="118"/>
+      <c r="B6" s="118"/>
+      <c r="C6" s="118"/>
+      <c r="D6" s="122"/>
+      <c r="E6" s="123"/>
+      <c r="F6" s="124"/>
     </row>
     <row r="7" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="28" t="s">
@@ -4626,13 +4212,13 @@
       <c r="A9" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="B9" s="110" t="s">
-        <v>91</v>
-      </c>
-      <c r="C9" s="111"/>
-      <c r="D9" s="111"/>
-      <c r="E9" s="111"/>
-      <c r="F9" s="112"/>
+      <c r="B9" s="146" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" s="147"/>
+      <c r="D9" s="147"/>
+      <c r="E9" s="147"/>
+      <c r="F9" s="148"/>
     </row>
     <row r="10" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="29" t="s">
@@ -4644,445 +4230,440 @@
       <c r="C10" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D10" s="134" t="s">
-        <v>62</v>
-      </c>
-      <c r="E10" s="134"/>
-      <c r="F10" s="134"/>
+      <c r="D10" s="117"/>
+      <c r="E10" s="117"/>
+      <c r="F10" s="117"/>
     </row>
     <row r="11" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="B11" s="113" t="s">
-        <v>92</v>
-      </c>
-      <c r="C11" s="114"/>
-      <c r="D11" s="114"/>
-      <c r="E11" s="114"/>
-      <c r="F11" s="115"/>
+        <v>62</v>
+      </c>
+      <c r="B11" s="149" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="150"/>
+      <c r="D11" s="150"/>
+      <c r="E11" s="150"/>
+      <c r="F11" s="151"/>
     </row>
     <row r="12" spans="1:7" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="49"/>
+      <c r="C12" s="110"/>
+      <c r="D12" s="110"/>
+      <c r="E12" s="110"/>
+      <c r="F12" s="110"/>
+    </row>
+    <row r="13" spans="1:7" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="110"/>
+      <c r="B13" s="110"/>
+      <c r="C13" s="110"/>
+      <c r="D13" s="110"/>
+      <c r="E13" s="110"/>
+      <c r="F13" s="110"/>
+    </row>
+    <row r="14" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="113" t="s">
         <v>64</v>
       </c>
-      <c r="B12" s="49"/>
-      <c r="C12" s="126"/>
-      <c r="D12" s="126"/>
-      <c r="E12" s="126"/>
-      <c r="F12" s="126"/>
-    </row>
-    <row r="13" spans="1:7" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="126"/>
-      <c r="B13" s="126"/>
-      <c r="C13" s="126"/>
-      <c r="D13" s="126"/>
-      <c r="E13" s="126"/>
-      <c r="F13" s="126"/>
-    </row>
-    <row r="14" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="130" t="s">
-        <v>65</v>
-      </c>
-      <c r="B14" s="130"/>
-      <c r="C14" s="130"/>
-      <c r="D14" s="130"/>
-      <c r="E14" s="130"/>
-      <c r="F14" s="130"/>
+      <c r="B14" s="113"/>
+      <c r="C14" s="113"/>
+      <c r="D14" s="113"/>
+      <c r="E14" s="113"/>
+      <c r="F14" s="113"/>
     </row>
     <row r="15" spans="1:7" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="23"/>
       <c r="B15" s="23"/>
       <c r="C15" s="23"/>
       <c r="D15" s="23"/>
-      <c r="E15" s="132"/>
-      <c r="F15" s="133"/>
+      <c r="E15" s="115"/>
+      <c r="F15" s="116"/>
     </row>
     <row r="16" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="24"/>
       <c r="B16" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="D16" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="E16" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="E16" s="131" t="s">
+      <c r="F16" s="114"/>
+    </row>
+    <row r="17" spans="1:9" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="F16" s="131"/>
-    </row>
-    <row r="17" spans="1:6" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="28" t="s">
-        <v>70</v>
-      </c>
       <c r="B17" s="52" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C17" s="41"/>
       <c r="D17" s="26"/>
-      <c r="E17" s="128"/>
-      <c r="F17" s="129"/>
-    </row>
-    <row r="18" spans="1:6" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E17" s="111"/>
+      <c r="F17" s="112"/>
+    </row>
+    <row r="18" spans="1:9" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="29" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B18" s="52" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C18" s="41"/>
       <c r="D18" s="26"/>
-      <c r="E18" s="128"/>
-      <c r="F18" s="129"/>
-    </row>
-    <row r="19" spans="1:6" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E18" s="111"/>
+      <c r="F18" s="112"/>
+    </row>
+    <row r="19" spans="1:9" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
       <c r="D19" s="26"/>
-      <c r="E19" s="128"/>
-      <c r="F19" s="129"/>
-    </row>
-    <row r="20" spans="1:6" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="126"/>
-      <c r="B20" s="126"/>
-      <c r="C20" s="126"/>
-      <c r="D20" s="126"/>
-      <c r="E20" s="126"/>
-      <c r="F20" s="126"/>
-    </row>
-    <row r="21" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="116" t="s">
+      <c r="E19" s="111"/>
+      <c r="F19" s="112"/>
+    </row>
+    <row r="20" spans="1:9" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="110"/>
+      <c r="B20" s="110"/>
+      <c r="C20" s="110"/>
+      <c r="D20" s="110"/>
+      <c r="E20" s="110"/>
+      <c r="F20" s="110"/>
+    </row>
+    <row r="21" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="126" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" s="127"/>
+      <c r="C21" s="127"/>
+      <c r="D21" s="127"/>
+      <c r="E21" s="127"/>
+      <c r="F21" s="128"/>
+    </row>
+    <row r="22" spans="1:9" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="107" t="s">
         <v>73</v>
       </c>
-      <c r="B21" s="117"/>
-      <c r="C21" s="117"/>
-      <c r="D21" s="117"/>
-      <c r="E21" s="117"/>
-      <c r="F21" s="118"/>
-    </row>
-    <row r="22" spans="1:6" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="119" t="s">
+      <c r="B22" s="108"/>
+      <c r="C22" s="53" t="s">
+        <v>107</v>
+      </c>
+      <c r="D22" s="53" t="s">
+        <v>109</v>
+      </c>
+      <c r="E22" s="105" t="s">
         <v>74</v>
       </c>
-      <c r="B22" s="120"/>
-      <c r="C22" s="120"/>
-      <c r="D22" s="120" t="s">
+      <c r="F22" s="106"/>
+    </row>
+    <row r="23" spans="1:9" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="103"/>
+      <c r="B23" s="104"/>
+      <c r="C23" s="55"/>
+      <c r="D23" s="55" t="s">
+        <v>97</v>
+      </c>
+      <c r="E23" s="103"/>
+      <c r="F23" s="104"/>
+    </row>
+    <row r="24" spans="1:9" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="103"/>
+      <c r="B24" s="104"/>
+      <c r="C24" s="55"/>
+      <c r="D24" s="55" t="s">
+        <v>104</v>
+      </c>
+      <c r="E24" s="103"/>
+      <c r="F24" s="104"/>
+    </row>
+    <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="103"/>
+      <c r="B25" s="104"/>
+      <c r="C25" s="55"/>
+      <c r="D25" s="55" t="s">
+        <v>104</v>
+      </c>
+      <c r="E25" s="103"/>
+      <c r="F25" s="104"/>
+    </row>
+    <row r="26" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="103"/>
+      <c r="B26" s="104"/>
+      <c r="C26" s="55"/>
+      <c r="D26" s="55"/>
+      <c r="E26" s="103"/>
+      <c r="F26" s="104"/>
+    </row>
+    <row r="27" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="103"/>
+      <c r="B27" s="104"/>
+      <c r="C27" s="55"/>
+      <c r="D27" s="55"/>
+      <c r="E27" s="103"/>
+      <c r="F27" s="104"/>
+    </row>
+    <row r="28" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="103"/>
+      <c r="B28" s="104"/>
+      <c r="C28" s="55"/>
+      <c r="D28" s="55"/>
+      <c r="E28" s="103"/>
+      <c r="F28" s="104"/>
+      <c r="I28" s="157"/>
+    </row>
+    <row r="29" spans="1:9" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="110"/>
+      <c r="B29" s="110"/>
+      <c r="C29" s="110"/>
+      <c r="D29" s="110"/>
+      <c r="E29" s="110"/>
+      <c r="F29" s="110"/>
+    </row>
+    <row r="30" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="126" t="s">
         <v>75</v>
       </c>
-      <c r="E22" s="120"/>
-      <c r="F22" s="121"/>
-    </row>
-    <row r="23" spans="1:6" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="100" t="s">
-        <v>102</v>
-      </c>
-      <c r="B23" s="100"/>
-      <c r="C23" s="100"/>
-      <c r="D23" s="100" t="s">
-        <v>101</v>
-      </c>
-      <c r="E23" s="100"/>
-      <c r="F23" s="100"/>
-    </row>
-    <row r="24" spans="1:6" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="100" t="s">
-        <v>109</v>
-      </c>
-      <c r="B24" s="100"/>
-      <c r="C24" s="100"/>
-      <c r="D24" s="100" t="s">
+      <c r="B30" s="127"/>
+      <c r="C30" s="127"/>
+      <c r="D30" s="127"/>
+      <c r="E30" s="127"/>
+      <c r="F30" s="128"/>
+    </row>
+    <row r="31" spans="1:9" ht="10.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="129" t="s">
+        <v>73</v>
+      </c>
+      <c r="B31" s="130"/>
+      <c r="C31" s="130"/>
+      <c r="D31" s="130" t="s">
+        <v>76</v>
+      </c>
+      <c r="E31" s="130"/>
+      <c r="F31" s="131"/>
+    </row>
+    <row r="32" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="125"/>
+      <c r="B32" s="125"/>
+      <c r="C32" s="125"/>
+      <c r="D32" s="125"/>
+      <c r="E32" s="125"/>
+      <c r="F32" s="125"/>
+    </row>
+    <row r="33" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="125"/>
+      <c r="B33" s="125"/>
+      <c r="C33" s="125"/>
+      <c r="D33" s="125"/>
+      <c r="E33" s="125"/>
+      <c r="F33" s="125"/>
+    </row>
+    <row r="34" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="125"/>
+      <c r="B34" s="125"/>
+      <c r="C34" s="125"/>
+      <c r="D34" s="125"/>
+      <c r="E34" s="125"/>
+      <c r="F34" s="125"/>
+    </row>
+    <row r="35" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="125"/>
+      <c r="B35" s="125"/>
+      <c r="C35" s="125"/>
+      <c r="D35" s="125"/>
+      <c r="E35" s="125"/>
+      <c r="F35" s="125"/>
+    </row>
+    <row r="36" spans="1:6" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="110"/>
+      <c r="B36" s="110"/>
+      <c r="C36" s="110"/>
+      <c r="D36" s="110"/>
+      <c r="E36" s="110"/>
+      <c r="F36" s="110"/>
+    </row>
+    <row r="37" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="126" t="s">
+        <v>77</v>
+      </c>
+      <c r="B37" s="127"/>
+      <c r="C37" s="127"/>
+      <c r="D37" s="127"/>
+      <c r="E37" s="127"/>
+      <c r="F37" s="128"/>
+    </row>
+    <row r="38" spans="1:6" ht="10.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="107" t="s">
+        <v>105</v>
+      </c>
+      <c r="B38" s="108"/>
+      <c r="C38" s="53" t="s">
+        <v>106</v>
+      </c>
+      <c r="D38" s="53" t="s">
+        <v>107</v>
+      </c>
+      <c r="E38" s="105" t="s">
+        <v>108</v>
+      </c>
+      <c r="F38" s="106"/>
+    </row>
+    <row r="39" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="103"/>
+      <c r="B39" s="104"/>
+      <c r="C39" s="54"/>
+      <c r="D39" s="54"/>
+      <c r="E39" s="134"/>
+      <c r="F39" s="135"/>
+    </row>
+    <row r="40" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="103"/>
+      <c r="B40" s="104"/>
+      <c r="C40" s="54"/>
+      <c r="D40" s="54"/>
+      <c r="E40" s="134"/>
+      <c r="F40" s="135"/>
+    </row>
+    <row r="41" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="103"/>
+      <c r="B41" s="104"/>
+      <c r="C41" s="54"/>
+      <c r="D41" s="54"/>
+      <c r="E41" s="134"/>
+      <c r="F41" s="135"/>
+    </row>
+    <row r="42" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="103"/>
+      <c r="B42" s="104"/>
+      <c r="C42" s="54"/>
+      <c r="D42" s="54"/>
+      <c r="E42" s="134"/>
+      <c r="F42" s="135"/>
+    </row>
+    <row r="43" spans="1:6" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="110"/>
+      <c r="B43" s="110"/>
+      <c r="C43" s="110"/>
+      <c r="D43" s="110"/>
+      <c r="E43" s="110"/>
+      <c r="F43" s="110"/>
+    </row>
+    <row r="44" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="126" t="s">
         <v>110</v>
       </c>
-      <c r="E24" s="100"/>
-      <c r="F24" s="100"/>
-    </row>
-    <row r="25" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A25" s="100" t="s">
-        <v>111</v>
-      </c>
-      <c r="B25" s="100"/>
-      <c r="C25" s="100"/>
-      <c r="D25" s="100" t="s">
-        <v>110</v>
-      </c>
-      <c r="E25" s="100"/>
-      <c r="F25" s="100"/>
-    </row>
-    <row r="26" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="100"/>
-      <c r="B26" s="100"/>
-      <c r="C26" s="100"/>
-      <c r="D26" s="100"/>
-      <c r="E26" s="100"/>
-      <c r="F26" s="100"/>
-    </row>
-    <row r="27" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="100"/>
-      <c r="B27" s="100"/>
-      <c r="C27" s="100"/>
-      <c r="D27" s="100"/>
-      <c r="E27" s="100"/>
-      <c r="F27" s="100"/>
-    </row>
-    <row r="28" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="100"/>
-      <c r="B28" s="100"/>
-      <c r="C28" s="100"/>
-      <c r="D28" s="100"/>
-      <c r="E28" s="100"/>
-      <c r="F28" s="100"/>
-    </row>
-    <row r="29" spans="1:6" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="126"/>
-      <c r="B29" s="126"/>
-      <c r="C29" s="126"/>
-      <c r="D29" s="126"/>
-      <c r="E29" s="126"/>
-      <c r="F29" s="126"/>
-    </row>
-    <row r="30" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="116" t="s">
-        <v>76</v>
-      </c>
-      <c r="B30" s="117"/>
-      <c r="C30" s="117"/>
-      <c r="D30" s="117"/>
-      <c r="E30" s="117"/>
-      <c r="F30" s="118"/>
-    </row>
-    <row r="31" spans="1:6" ht="10.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="119" t="s">
-        <v>74</v>
-      </c>
-      <c r="B31" s="120"/>
-      <c r="C31" s="120"/>
-      <c r="D31" s="120" t="s">
-        <v>77</v>
-      </c>
-      <c r="E31" s="120"/>
-      <c r="F31" s="121"/>
-    </row>
-    <row r="32" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="100"/>
-      <c r="B32" s="100"/>
-      <c r="C32" s="100"/>
-      <c r="D32" s="100"/>
-      <c r="E32" s="100"/>
-      <c r="F32" s="100"/>
-    </row>
-    <row r="33" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="100"/>
-      <c r="B33" s="100"/>
-      <c r="C33" s="100"/>
-      <c r="D33" s="100"/>
-      <c r="E33" s="100"/>
-      <c r="F33" s="100"/>
-    </row>
-    <row r="34" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="100"/>
-      <c r="B34" s="100"/>
-      <c r="C34" s="100"/>
-      <c r="D34" s="100"/>
-      <c r="E34" s="100"/>
-      <c r="F34" s="100"/>
-    </row>
-    <row r="35" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="100"/>
-      <c r="B35" s="100"/>
-      <c r="C35" s="100"/>
-      <c r="D35" s="100"/>
-      <c r="E35" s="100"/>
-      <c r="F35" s="100"/>
-    </row>
-    <row r="36" spans="1:6" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="126"/>
-      <c r="B36" s="126"/>
-      <c r="C36" s="126"/>
-      <c r="D36" s="126"/>
-      <c r="E36" s="126"/>
-      <c r="F36" s="126"/>
-    </row>
-    <row r="37" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="116" t="s">
-        <v>78</v>
-      </c>
-      <c r="B37" s="117"/>
-      <c r="C37" s="117"/>
-      <c r="D37" s="117"/>
-      <c r="E37" s="117"/>
-      <c r="F37" s="118"/>
-    </row>
-    <row r="38" spans="1:6" ht="10.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="B38" s="120" t="s">
-        <v>74</v>
-      </c>
-      <c r="C38" s="120"/>
-      <c r="D38" s="120"/>
-      <c r="E38" s="120" t="s">
-        <v>80</v>
-      </c>
-      <c r="F38" s="121"/>
-    </row>
-    <row r="39" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="27"/>
-      <c r="B39" s="122" t="s">
-        <v>88</v>
-      </c>
-      <c r="C39" s="122"/>
-      <c r="D39" s="122"/>
-      <c r="E39" s="123"/>
-      <c r="F39" s="123"/>
-    </row>
-    <row r="40" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="27"/>
-      <c r="B40" s="122" t="s">
-        <v>89</v>
-      </c>
-      <c r="C40" s="122"/>
-      <c r="D40" s="122"/>
-      <c r="E40" s="123"/>
-      <c r="F40" s="123"/>
-    </row>
-    <row r="41" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="27"/>
-      <c r="B41" s="122"/>
-      <c r="C41" s="122"/>
-      <c r="D41" s="122"/>
-      <c r="E41" s="123"/>
-      <c r="F41" s="123"/>
-    </row>
-    <row r="42" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="27"/>
-      <c r="B42" s="122"/>
-      <c r="C42" s="122"/>
-      <c r="D42" s="122"/>
-      <c r="E42" s="123"/>
-      <c r="F42" s="123"/>
-    </row>
-    <row r="43" spans="1:6" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="126"/>
-      <c r="B43" s="126"/>
-      <c r="C43" s="126"/>
-      <c r="D43" s="126"/>
-      <c r="E43" s="126"/>
-      <c r="F43" s="126"/>
-    </row>
-    <row r="44" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="116" t="s">
-        <v>81</v>
-      </c>
-      <c r="B44" s="117"/>
-      <c r="C44" s="117"/>
-      <c r="D44" s="117"/>
-      <c r="E44" s="117"/>
-      <c r="F44" s="118"/>
+      <c r="B44" s="127"/>
+      <c r="C44" s="127"/>
+      <c r="D44" s="127"/>
+      <c r="E44" s="127"/>
+      <c r="F44" s="128"/>
     </row>
     <row r="45" spans="1:6" ht="10.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="31" t="s">
+        <v>78</v>
+      </c>
+      <c r="B45" s="130" t="s">
+        <v>73</v>
+      </c>
+      <c r="C45" s="130"/>
+      <c r="D45" s="130"/>
+      <c r="E45" s="130" t="s">
         <v>79</v>
       </c>
-      <c r="B45" s="120" t="s">
-        <v>74</v>
-      </c>
-      <c r="C45" s="120"/>
-      <c r="D45" s="120"/>
-      <c r="E45" s="120" t="s">
-        <v>80</v>
-      </c>
-      <c r="F45" s="121"/>
+      <c r="F45" s="131"/>
     </row>
     <row r="46" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="27" t="s">
-        <v>104</v>
-      </c>
-      <c r="B46" s="122" t="s">
-        <v>103</v>
-      </c>
-      <c r="C46" s="122"/>
-      <c r="D46" s="122"/>
-      <c r="E46" s="123">
+        <v>99</v>
+      </c>
+      <c r="B46" s="118" t="s">
+        <v>98</v>
+      </c>
+      <c r="C46" s="118"/>
+      <c r="D46" s="118"/>
+      <c r="E46" s="132">
         <v>6</v>
       </c>
-      <c r="F46" s="123"/>
+      <c r="F46" s="132"/>
     </row>
     <row r="47" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="B47" s="122" t="s">
-        <v>105</v>
-      </c>
-      <c r="C47" s="122"/>
-      <c r="D47" s="122"/>
-      <c r="E47" s="123">
+        <v>101</v>
+      </c>
+      <c r="B47" s="118" t="s">
+        <v>100</v>
+      </c>
+      <c r="C47" s="118"/>
+      <c r="D47" s="118"/>
+      <c r="E47" s="132">
         <v>1</v>
       </c>
-      <c r="F47" s="123"/>
+      <c r="F47" s="132"/>
     </row>
     <row r="48" spans="1:6" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="B48" s="122" t="s">
-        <v>108</v>
-      </c>
-      <c r="C48" s="122"/>
-      <c r="D48" s="122"/>
-      <c r="E48" s="123">
+        <v>102</v>
+      </c>
+      <c r="B48" s="118" t="s">
+        <v>103</v>
+      </c>
+      <c r="C48" s="118"/>
+      <c r="D48" s="118"/>
+      <c r="E48" s="132">
         <v>12</v>
       </c>
-      <c r="F48" s="123"/>
+      <c r="F48" s="132"/>
     </row>
     <row r="49" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="27"/>
-      <c r="B49" s="122"/>
-      <c r="C49" s="122"/>
-      <c r="D49" s="122"/>
-      <c r="E49" s="123"/>
-      <c r="F49" s="123"/>
+      <c r="B49" s="118"/>
+      <c r="C49" s="118"/>
+      <c r="D49" s="118"/>
+      <c r="E49" s="132"/>
+      <c r="F49" s="132"/>
     </row>
     <row r="50" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="27"/>
-      <c r="B50" s="122"/>
-      <c r="C50" s="122"/>
-      <c r="D50" s="122"/>
-      <c r="E50" s="123"/>
-      <c r="F50" s="123"/>
+      <c r="B50" s="118"/>
+      <c r="C50" s="118"/>
+      <c r="D50" s="118"/>
+      <c r="E50" s="132"/>
+      <c r="F50" s="132"/>
     </row>
     <row r="51" spans="1:6" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="125"/>
-      <c r="B51" s="125"/>
-      <c r="C51" s="125"/>
-      <c r="D51" s="125"/>
-      <c r="E51" s="125"/>
-      <c r="F51" s="125"/>
+      <c r="A51" s="136"/>
+      <c r="B51" s="136"/>
+      <c r="C51" s="136"/>
+      <c r="D51" s="136"/>
+      <c r="E51" s="136"/>
+      <c r="F51" s="136"/>
     </row>
     <row r="52" spans="1:6" ht="62.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="123" t="s">
-        <v>82</v>
-      </c>
-      <c r="B52" s="123"/>
-      <c r="C52" s="123"/>
-      <c r="D52" s="123"/>
-      <c r="E52" s="123"/>
-      <c r="F52" s="123"/>
+      <c r="A52" s="132" t="s">
+        <v>80</v>
+      </c>
+      <c r="B52" s="132"/>
+      <c r="C52" s="132"/>
+      <c r="D52" s="132"/>
+      <c r="E52" s="132"/>
+      <c r="F52" s="132"/>
     </row>
     <row r="53" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="124"/>
-      <c r="B53" s="124"/>
-      <c r="C53" s="124"/>
-      <c r="D53" s="124"/>
-      <c r="E53" s="124"/>
-      <c r="F53" s="124"/>
+      <c r="A53" s="133"/>
+      <c r="B53" s="133"/>
+      <c r="C53" s="133"/>
+      <c r="D53" s="133"/>
+      <c r="E53" s="133"/>
+      <c r="F53" s="133"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C55" s="20"/>
@@ -5090,6 +4671,51 @@
   </sheetData>
   <sheetProtection formatCells="0"/>
   <mergeCells count="72">
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="D2:F4"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="A43:F43"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A52:F52"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="E48:F48"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="D35:F35"/>
+    <mergeCell ref="A33:C33"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A20:F20"/>
     <mergeCell ref="E19:F19"/>
@@ -5103,65 +4729,20 @@
     <mergeCell ref="D10:F10"/>
     <mergeCell ref="A2:C6"/>
     <mergeCell ref="D5:F6"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="D32:F32"/>
-    <mergeCell ref="D33:F33"/>
-    <mergeCell ref="D34:F34"/>
-    <mergeCell ref="D35:F35"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="E50:F50"/>
-    <mergeCell ref="A53:F53"/>
-    <mergeCell ref="B38:D38"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="A51:F51"/>
-    <mergeCell ref="A52:F52"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="B48:D48"/>
-    <mergeCell ref="E48:F48"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="E49:F49"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="A43:F43"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="A44:F44"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="D2:F4"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
   </mergeCells>
   <pageMargins left="0.52999994886203072" right="0.52999994886203072" top="0.52999994886203072" bottom="0.68999998212799307" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="91" orientation="portrait" r:id="rId1"/>
@@ -5190,20 +4771,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
     </row>
     <row r="2" spans="1:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
@@ -5222,380 +4803,341 @@
       <c r="L2" s="18"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="144" t="s">
-        <v>74</v>
-      </c>
-      <c r="B3" s="145"/>
-      <c r="C3" s="145"/>
+      <c r="A3" s="152" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="153"/>
+      <c r="C3" s="153"/>
       <c r="D3" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="E3" s="144" t="s">
-        <v>74</v>
-      </c>
-      <c r="F3" s="145"/>
-      <c r="G3" s="145"/>
+      <c r="E3" s="152" t="s">
+        <v>73</v>
+      </c>
+      <c r="F3" s="153"/>
+      <c r="G3" s="153"/>
       <c r="H3" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="I3" s="144" t="s">
-        <v>74</v>
-      </c>
-      <c r="J3" s="145"/>
-      <c r="K3" s="145"/>
+      <c r="I3" s="152" t="s">
+        <v>73</v>
+      </c>
+      <c r="J3" s="153"/>
+      <c r="K3" s="153"/>
       <c r="L3" s="32" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="100" t="s">
-        <v>86</v>
-      </c>
-      <c r="B4" s="100"/>
-      <c r="C4" s="100"/>
+      <c r="A4" s="125" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4" s="125"/>
+      <c r="C4" s="125"/>
       <c r="D4" s="33">
         <v>46113</v>
       </c>
-      <c r="E4" s="100" t="s">
-        <v>87</v>
-      </c>
-      <c r="F4" s="100"/>
-      <c r="G4" s="100"/>
+      <c r="E4" s="125" t="s">
+        <v>85</v>
+      </c>
+      <c r="F4" s="125"/>
+      <c r="G4" s="125"/>
       <c r="H4" s="33">
         <v>46113</v>
       </c>
-      <c r="I4" s="122"/>
-      <c r="J4" s="122"/>
-      <c r="K4" s="122"/>
+      <c r="I4" s="118"/>
+      <c r="J4" s="118"/>
+      <c r="K4" s="118"/>
       <c r="L4" s="33"/>
     </row>
     <row r="5" spans="1:12" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="143" t="s">
-        <v>83</v>
-      </c>
-      <c r="B5" s="143"/>
-      <c r="C5" s="143"/>
-      <c r="D5" s="143"/>
-      <c r="E5" s="143"/>
-      <c r="F5" s="143"/>
-      <c r="G5" s="143"/>
-      <c r="H5" s="143"/>
-      <c r="I5" s="143"/>
-      <c r="J5" s="143"/>
-      <c r="K5" s="143"/>
-      <c r="L5" s="143"/>
+      <c r="A5" s="154" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="154"/>
+      <c r="C5" s="154"/>
+      <c r="D5" s="154"/>
+      <c r="E5" s="154"/>
+      <c r="F5" s="154"/>
+      <c r="G5" s="154"/>
+      <c r="H5" s="154"/>
+      <c r="I5" s="154"/>
+      <c r="J5" s="154"/>
+      <c r="K5" s="154"/>
+      <c r="L5" s="154"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="B6" s="142"/>
-      <c r="C6" s="142"/>
+      <c r="A6" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="156"/>
+      <c r="C6" s="156"/>
       <c r="D6" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="E6" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="F6" s="142"/>
-      <c r="G6" s="142"/>
+      <c r="E6" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="F6" s="156"/>
+      <c r="G6" s="156"/>
       <c r="H6" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="I6" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="J6" s="142"/>
-      <c r="K6" s="142"/>
+      <c r="I6" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="J6" s="156"/>
+      <c r="K6" s="156"/>
       <c r="L6" s="34" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="122"/>
-      <c r="B7" s="122"/>
-      <c r="C7" s="122"/>
+      <c r="A7" s="118"/>
+      <c r="B7" s="118"/>
+      <c r="C7" s="118"/>
       <c r="D7" s="33"/>
-      <c r="E7" s="122"/>
-      <c r="F7" s="122"/>
-      <c r="G7" s="122"/>
+      <c r="E7" s="118"/>
+      <c r="F7" s="118"/>
+      <c r="G7" s="118"/>
       <c r="H7" s="33"/>
-      <c r="I7" s="122"/>
-      <c r="J7" s="122"/>
-      <c r="K7" s="122"/>
+      <c r="I7" s="118"/>
+      <c r="J7" s="118"/>
+      <c r="K7" s="118"/>
       <c r="L7" s="33"/>
     </row>
     <row r="8" spans="1:12" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="143"/>
-      <c r="B8" s="143"/>
-      <c r="C8" s="143"/>
-      <c r="D8" s="143"/>
-      <c r="E8" s="143"/>
-      <c r="F8" s="143"/>
-      <c r="G8" s="143"/>
-      <c r="H8" s="143"/>
-      <c r="I8" s="143"/>
-      <c r="J8" s="143"/>
-      <c r="K8" s="143"/>
-      <c r="L8" s="143"/>
+      <c r="A8" s="154"/>
+      <c r="B8" s="154"/>
+      <c r="C8" s="154"/>
+      <c r="D8" s="154"/>
+      <c r="E8" s="154"/>
+      <c r="F8" s="154"/>
+      <c r="G8" s="154"/>
+      <c r="H8" s="154"/>
+      <c r="I8" s="154"/>
+      <c r="J8" s="154"/>
+      <c r="K8" s="154"/>
+      <c r="L8" s="154"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="B9" s="142"/>
-      <c r="C9" s="142"/>
+      <c r="A9" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="156"/>
+      <c r="C9" s="156"/>
       <c r="D9" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="E9" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="F9" s="142"/>
-      <c r="G9" s="142"/>
+      <c r="E9" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="F9" s="156"/>
+      <c r="G9" s="156"/>
       <c r="H9" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="I9" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="J9" s="142"/>
-      <c r="K9" s="142"/>
+      <c r="I9" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="J9" s="156"/>
+      <c r="K9" s="156"/>
       <c r="L9" s="34" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="122"/>
-      <c r="B10" s="122"/>
-      <c r="C10" s="122"/>
+      <c r="A10" s="118"/>
+      <c r="B10" s="118"/>
+      <c r="C10" s="118"/>
       <c r="D10" s="33"/>
-      <c r="E10" s="122"/>
-      <c r="F10" s="122"/>
-      <c r="G10" s="122"/>
+      <c r="E10" s="118"/>
+      <c r="F10" s="118"/>
+      <c r="G10" s="118"/>
       <c r="H10" s="33"/>
-      <c r="I10" s="122"/>
-      <c r="J10" s="122"/>
-      <c r="K10" s="122"/>
+      <c r="I10" s="118"/>
+      <c r="J10" s="118"/>
+      <c r="K10" s="118"/>
       <c r="L10" s="33"/>
     </row>
     <row r="11" spans="1:12" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="143"/>
-      <c r="B11" s="143"/>
-      <c r="C11" s="143"/>
-      <c r="D11" s="143"/>
-      <c r="E11" s="143"/>
-      <c r="F11" s="143"/>
-      <c r="G11" s="143"/>
-      <c r="H11" s="143"/>
-      <c r="I11" s="143"/>
-      <c r="J11" s="143"/>
-      <c r="K11" s="143"/>
-      <c r="L11" s="143"/>
+      <c r="A11" s="154"/>
+      <c r="B11" s="154"/>
+      <c r="C11" s="154"/>
+      <c r="D11" s="154"/>
+      <c r="E11" s="154"/>
+      <c r="F11" s="154"/>
+      <c r="G11" s="154"/>
+      <c r="H11" s="154"/>
+      <c r="I11" s="154"/>
+      <c r="J11" s="154"/>
+      <c r="K11" s="154"/>
+      <c r="L11" s="154"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="B12" s="142"/>
-      <c r="C12" s="142"/>
+      <c r="A12" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="156"/>
+      <c r="C12" s="156"/>
       <c r="D12" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="E12" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="F12" s="142"/>
-      <c r="G12" s="142"/>
+      <c r="E12" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="F12" s="156"/>
+      <c r="G12" s="156"/>
       <c r="H12" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="I12" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="J12" s="142"/>
-      <c r="K12" s="142"/>
+      <c r="I12" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="J12" s="156"/>
+      <c r="K12" s="156"/>
       <c r="L12" s="34" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="122"/>
-      <c r="B13" s="122"/>
-      <c r="C13" s="122"/>
+      <c r="A13" s="118"/>
+      <c r="B13" s="118"/>
+      <c r="C13" s="118"/>
       <c r="D13" s="33"/>
-      <c r="E13" s="122"/>
-      <c r="F13" s="122"/>
-      <c r="G13" s="122"/>
+      <c r="E13" s="118"/>
+      <c r="F13" s="118"/>
+      <c r="G13" s="118"/>
       <c r="H13" s="33"/>
-      <c r="I13" s="122"/>
-      <c r="J13" s="122"/>
-      <c r="K13" s="122"/>
+      <c r="I13" s="118"/>
+      <c r="J13" s="118"/>
+      <c r="K13" s="118"/>
       <c r="L13" s="33"/>
     </row>
     <row r="14" spans="1:12" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="143"/>
-      <c r="B14" s="143"/>
-      <c r="C14" s="143"/>
-      <c r="D14" s="143"/>
-      <c r="E14" s="143"/>
-      <c r="F14" s="143"/>
-      <c r="G14" s="143"/>
-      <c r="H14" s="143"/>
-      <c r="I14" s="143"/>
-      <c r="J14" s="143"/>
-      <c r="K14" s="143"/>
-      <c r="L14" s="143"/>
+      <c r="A14" s="154"/>
+      <c r="B14" s="154"/>
+      <c r="C14" s="154"/>
+      <c r="D14" s="154"/>
+      <c r="E14" s="154"/>
+      <c r="F14" s="154"/>
+      <c r="G14" s="154"/>
+      <c r="H14" s="154"/>
+      <c r="I14" s="154"/>
+      <c r="J14" s="154"/>
+      <c r="K14" s="154"/>
+      <c r="L14" s="154"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="B15" s="142"/>
-      <c r="C15" s="142"/>
+      <c r="A15" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="156"/>
+      <c r="C15" s="156"/>
       <c r="D15" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="E15" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="F15" s="142"/>
-      <c r="G15" s="142"/>
+      <c r="E15" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="F15" s="156"/>
+      <c r="G15" s="156"/>
       <c r="H15" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="I15" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="J15" s="142"/>
-      <c r="K15" s="142"/>
+      <c r="I15" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="J15" s="156"/>
+      <c r="K15" s="156"/>
       <c r="L15" s="34" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="122"/>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
+      <c r="A16" s="118"/>
+      <c r="B16" s="118"/>
+      <c r="C16" s="118"/>
       <c r="D16" s="33"/>
-      <c r="E16" s="122"/>
-      <c r="F16" s="122"/>
-      <c r="G16" s="122"/>
+      <c r="E16" s="118"/>
+      <c r="F16" s="118"/>
+      <c r="G16" s="118"/>
       <c r="H16" s="33"/>
-      <c r="I16" s="122"/>
-      <c r="J16" s="122"/>
-      <c r="K16" s="122"/>
+      <c r="I16" s="118"/>
+      <c r="J16" s="118"/>
+      <c r="K16" s="118"/>
       <c r="L16" s="33"/>
     </row>
     <row r="17" spans="1:12" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="143"/>
-      <c r="B17" s="143"/>
-      <c r="C17" s="143"/>
-      <c r="D17" s="143"/>
-      <c r="E17" s="143"/>
-      <c r="F17" s="143"/>
-      <c r="G17" s="143"/>
-      <c r="H17" s="143"/>
-      <c r="I17" s="143"/>
-      <c r="J17" s="143"/>
-      <c r="K17" s="143"/>
-      <c r="L17" s="143"/>
+      <c r="A17" s="154"/>
+      <c r="B17" s="154"/>
+      <c r="C17" s="154"/>
+      <c r="D17" s="154"/>
+      <c r="E17" s="154"/>
+      <c r="F17" s="154"/>
+      <c r="G17" s="154"/>
+      <c r="H17" s="154"/>
+      <c r="I17" s="154"/>
+      <c r="J17" s="154"/>
+      <c r="K17" s="154"/>
+      <c r="L17" s="154"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A18" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="B18" s="142"/>
-      <c r="C18" s="142"/>
+      <c r="A18" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18" s="156"/>
+      <c r="C18" s="156"/>
       <c r="D18" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="E18" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="F18" s="142"/>
-      <c r="G18" s="142"/>
+      <c r="E18" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="F18" s="156"/>
+      <c r="G18" s="156"/>
       <c r="H18" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="I18" s="141" t="s">
-        <v>74</v>
-      </c>
-      <c r="J18" s="142"/>
-      <c r="K18" s="142"/>
+      <c r="I18" s="155" t="s">
+        <v>73</v>
+      </c>
+      <c r="J18" s="156"/>
+      <c r="K18" s="156"/>
       <c r="L18" s="34" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="122"/>
-      <c r="B19" s="122"/>
-      <c r="C19" s="122"/>
+      <c r="A19" s="118"/>
+      <c r="B19" s="118"/>
+      <c r="C19" s="118"/>
       <c r="D19" s="33"/>
-      <c r="E19" s="122"/>
-      <c r="F19" s="122"/>
-      <c r="G19" s="122"/>
+      <c r="E19" s="118"/>
+      <c r="F19" s="118"/>
+      <c r="G19" s="118"/>
       <c r="H19" s="33"/>
-      <c r="I19" s="122"/>
-      <c r="J19" s="122"/>
-      <c r="K19" s="122"/>
+      <c r="I19" s="118"/>
+      <c r="J19" s="118"/>
+      <c r="K19" s="118"/>
       <c r="L19" s="33"/>
     </row>
     <row r="20" spans="1:12" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="143"/>
-      <c r="B20" s="143"/>
-      <c r="C20" s="143"/>
-      <c r="D20" s="143"/>
-      <c r="E20" s="143"/>
-      <c r="F20" s="143"/>
-      <c r="G20" s="143"/>
-      <c r="H20" s="143"/>
-      <c r="I20" s="143"/>
-      <c r="J20" s="143"/>
-      <c r="K20" s="143"/>
-      <c r="L20" s="143"/>
+      <c r="A20" s="154"/>
+      <c r="B20" s="154"/>
+      <c r="C20" s="154"/>
+      <c r="D20" s="154"/>
+      <c r="E20" s="154"/>
+      <c r="F20" s="154"/>
+      <c r="G20" s="154"/>
+      <c r="H20" s="154"/>
+      <c r="I20" s="154"/>
+      <c r="J20" s="154"/>
+      <c r="K20" s="154"/>
+      <c r="L20" s="154"/>
     </row>
   </sheetData>
   <mergeCells count="55">
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="I3:K3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="I5:L5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="I6:K6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="I8:L8"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="E11:H11"/>
-    <mergeCell ref="I11:L11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="E12:G12"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="E20:H20"/>
-    <mergeCell ref="I20:L20"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="E14:H14"/>
-    <mergeCell ref="I14:L14"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="E18:G18"/>
@@ -5612,18 +5154,59 @@
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="I15:K15"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="E20:H20"/>
+    <mergeCell ref="I20:L20"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="E14:H14"/>
+    <mergeCell ref="I14:L14"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="E11:H11"/>
+    <mergeCell ref="I11:L11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="I8:L8"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="I5:L5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="I6:K6"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="I4:K4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="949e891a-c427-49d3-9aba-de49c1d1085f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e5f17793-c322-4a32-a62c-554e3c75c14e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5862,20 +5445,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="949e891a-c427-49d3-9aba-de49c1d1085f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e5f17793-c322-4a32-a62c-554e3c75c14e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB4B6772-D837-4FE5-B5FF-A19CEF8AF4C0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE17DA02-B7E4-4CE0-B7FD-4CDC1788686E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="949e891a-c427-49d3-9aba-de49c1d1085f"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="e5f17793-c322-4a32-a62c-554e3c75c14e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5900,18 +5490,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE17DA02-B7E4-4CE0-B7FD-4CDC1788686E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB4B6772-D837-4FE5-B5FF-A19CEF8AF4C0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="949e891a-c427-49d3-9aba-de49c1d1085f"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="e5f17793-c322-4a32-a62c-554e3c75c14e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update RDO team quantity label
</commit_message>
<xml_diff>
--- a/assets/templates/modelo-de-diario-de-obras-2-0.xlsx
+++ b/assets/templates/modelo-de-diario-de-obras-2-0.xlsx
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="112">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -552,6 +552,9 @@
   </si>
   <si>
     <t>Materiais utilizados</t>
+  </si>
+  <si>
+    <t>Quantidade de funcionários</t>
   </si>
 </sst>
 </file>
@@ -4507,7 +4510,7 @@
       </c>
       <c r="B38" s="108"/>
       <c r="C38" s="53" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D38" s="53" t="s">
         <v>107</v>

</xml_diff>